<commit_message>
Apply Claude-validated corrections to Program_Spec_Workbook.xlsx
7 corrections applied after validating GPT review against actual R code:

1. SCT tandem AUTO: Added >=60 day lower bound to definition (was <=180 only)
2. LOT1_1ST_SCT_DT: Fixed formula from min(AUTO_DT_1, TX_ENDDATE) to
   least(AUTO_DT_1, FIRST_ALLO_DT, FIRST_CART_DT) per code lines 3963-3972
3. DAY_SUPPLY: Flagged protocol mismatch - code deletes pharmacy claims with
   missing/<1 DAY_SUPPLY but protocol says default to 28 days (NYY status)
4. ENDDATE in lot1base: Updated to document OBS_END_DT usage per code
5. LOT1_BASE_LENGTH: Added missing add-med third branch to definition
6-7. Add-med tie-break: Updated from 'random' to deterministic min(MAP_MED_TYPE)

GPT review issues NOT applied (inaccurate):
- Exclusion toggle defaults claimed FALSE but are TRUE in interactive mode
- Other cancer window claim conflated 30-day pair-matching with outpatient_window

https://claude.ai/code/session_01K25gca9CxWw3eVA3yixKC5
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/Program_Spec_Workbook.xlsx
+++ b/docs/Part 3/Program Spec/Program_Spec_Workbook.xlsx
@@ -2070,7 +2070,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -2567,7 +2566,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -3002,7 +3000,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -3747,7 +3744,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -4182,7 +4178,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -5051,7 +5046,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -5672,7 +5666,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -6355,7 +6348,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -7280,7 +7272,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -7459,7 +7450,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The end date of a patient's observation period, defined as the earliest of death, health plan disenrollment, or the end of the study period (30 June 2025). Merged from the ELIG_COH dataset via PAT_ID.</t>
+          <t>The end date of a patient's observation period, defined as the earliest of death, health plan disenrollment, or the end of the study period (30 June 2025). Merged from the ELIG_COH dataset via PAT_ID. NOTE: In the R code, the LOT logic uses OBS_END_DT = coalesce(ENDDATE_CE, ENDDATE) rather than raw ENDDATE. ENDDATE_CE properly accounts for disenrollment gaps while raw ENDDATE may extend beyond disenrollment. All LOT1 boundary calculations (discontinuation, add-med, SCT, censoring) use OBS_END_DT.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -7479,17 +7470,22 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>YYN</t>
+          <t>YYY</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Spec=Y: matches protocol definition. Protocol=Y: correctly defines observation end. Code=N: Code uses OBS_END_DT (coalesce of ENDDATE_CE and ENDDATE) rather than raw ENDDATE. This is a refinement - ENDDATE_CE properly accounts for disenrollment gaps while ENDDATE may extend beyond disenrollment. The code is more conservative/correct than the spec's simple ENDDATE reference.</t>
+          <t>Spec=Y: Now correctly documents OBS_END_DT usage. Protocol=Y: correctly defines observation end. Code=Y: Uses OBS_END_DT = coalesce(ENDDATE_CE, ENDDATE) for all LOT logic (lot_program.R line 2899).</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Claude Review 2026-03-18</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Minor discrepancy: Spec says 'merge ENDDATE from ELIG_COH' but the R code actually uses OBS_END_DT = coalesce(ENDDATE_CE, ENDDATE) which is more precise. ENDDATE_CE incorporates disenrollment end dates. This is a deliberate code improvement over the spec but creates a spec-code mismatch.</t>
+          <t>RESOLVED: Previously, spec referenced raw ENDDATE but code uses OBS_END_DT = coalesce(ENDDATE_CE, ENDDATE). Definition now documents OBS_END_DT usage. This is a code improvement over the original spec, properly accounting for disenrollment.</t>
         </is>
       </c>
     </row>
@@ -7823,7 +7819,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The number of days of the LOT1 Base period. If LOT1_BASE_DISCON_DT is not missing: LOT1_BASE_DISCON_DT - LOT1_START_DT + 1. If LOT1_BASE_DISCON_DT is missing: ENDDATE - LOT1_START_DT + 1.</t>
+          <t>The number of days of the LOT1 Base period. Calculated with three-way priority: (1) If LOT1_BASE_1ST_ADD_MED_DT is not missing AND (LOT1_BASE_DISCON_DT is missing OR LOT1_BASE_1ST_ADD_MED_DT &lt;= LOT1_BASE_DISCON_DT): LOT1_BASE_1ST_ADD_MED_DT - LOT1_START_DT + 1. (2) If LOT1_BASE_DISCON_DT is not missing: LOT1_BASE_DISCON_DT - LOT1_START_DT + 1. (3) Otherwise (censored): OBS_END_DT - LOT1_START_DT + 1.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -7843,17 +7839,22 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>YYY</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Spec=N: Spec only considers two cases (discon_dt present or missing). Protocol=Y: LOT end includes medication add as a terminating event. Code=Y: Correctly handles three cases: (1) add-med ends base before discon, (2) discon ends base, (3) fallback to OBS_END_DT.</t>
+          <t>Spec=Y: Now correctly defines three-way priority (add-med &gt; discon &gt; censored). Protocol=Y: LOT end includes medication add as a terminating event per Section 5.1.1. Code=Y: Implements three-way CASE at lot_program.R lines 3447-3455.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Claude Review 2026-03-18</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Discrepancy: The spec defines LOT1_BASE_LENGTH with only two branches (discon present vs missing) but does not account for the LOT1_BASE_1ST_ADD_MED_DT case. The R code correctly adds a third branch: if a new medication is added (LOT1_BASE_1ST_ADD_MED_DT) before discontinuation, the base period ends at the add-med date. This is consistent with the protocol (Section 5.1.1 item 1: substitution of a new MM treatment ends the LOT). The spec is incomplete.</t>
+          <t>RESOLVED: Previously only had two branches (discon present vs missing), missing the add-med case. Now includes three-way priority matching code: (1) add-med ends base before discon, (2) discon ends base, (3) fallback to OBS_END_DT.</t>
         </is>
       </c>
     </row>
@@ -7875,7 +7876,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The day before the earliest MAP_START_DT of a medication [MED] that is NOT in LOT1_BASE_MEDS (and is not a permissible substitution), where MAP_START_DT falls between LOT1_START_DT and LOT1_BASE_DISCON_DT (or OBS_END_DT if discon is missing). If multiple [MED]s on the same earliest date, one is selected (spec says random; code uses min for determinism). Set to missing if no such MAPs are found.</t>
+          <t>The day before the earliest MAP_START_DT of a medication [MED] that is NOT in LOT1_BASE_MEDS (and is not a permissible substitution), where MAP_START_DT falls between LOT1_START_DT and LOT1_BASE_DISCON_DT (or OBS_END_DT if discon is missing). If multiple [MED]s on the same earliest date, the one with the alphabetically first MAP_MED_TYPE is selected (deterministic via min(MAP_MED_TYPE) for reproducibility). Set to missing if no such MAPs are found.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -7895,17 +7896,22 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>YYN</t>
+          <t>YYY</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Spec=Y: Correctly defines as day before earliest non-base-med MAP. Protocol=Y: Matches Section 5.1.1 new agent rule. Code=N (minor): Code uses min(MAP_MED_TYPE) for same-day ties instead of random selection as spec states. This is a deliberate, documented deviation for reproducibility.</t>
+          <t>Spec=Y: Now documents deterministic tie-break (min(MAP_MED_TYPE)). Protocol=Y: Protocol does not specify tie-breaking method. Code=Y: Uses min(MAP_MED_TYPE) at lot_program.R line 3435 with explicit comment about deliberate deviation from original random spec.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Claude Review 2026-03-18</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Minor discrepancy: Spec states 'select one of them at random' for same-day ties. Code uses min(MAP_MED_TYPE) instead for deterministic results (documented at line 3435). The MAP_MED_TYPE selection only affects LOT1_BASE_1ST_ADD_MED name, not the date. This is a reasonable implementation choice for reproducibility.</t>
+          <t>RESOLVED: Updated from 'random' to deterministic min(MAP_MED_TYPE) to match code implementation. This is a deliberate deviation for reproducibility (code comment at line 3435). The selection only affects the medication NAME, not the date.</t>
         </is>
       </c>
     </row>
@@ -7947,17 +7953,22 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>YYN</t>
+          <t>YYY</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Spec=Y: Correctly defined as medication name from add-med logic. Protocol=Y: Implicit in LOT transition rules. Code=N (minor): Uses min() instead of random for tie-breaking, same as LOT1_BASE_1ST_ADD_MED_DT deviation.</t>
+          <t>Spec=Y: Correctly defined as medication name from add-med logic with deterministic tie-break. Protocol=Y: Implicit in LOT transition rules. Code=Y: Uses min(MAP_MED_TYPE) at lot_program.R line 3436.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Claude Review 2026-03-18</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Minor discrepancy: Same tie-breaking deviation as LOT1_BASE_1ST_ADD_MED_DT - code uses min() instead of random. See LOT1_BASE_1ST_ADD_MED_DT row for details.</t>
+          <t>RESOLVED: Same deterministic tie-break fix as LOT1_BASE_1ST_ADD_MED_DT.</t>
         </is>
       </c>
     </row>
@@ -18455,17 +18466,22 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>YYY</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Spec: Y - correctly defines DATE_SERVICE as the service date filtered between INDEX_DATE and ENDDATE inclusive, with proper dedup rules. Protocol: Y - confirms observation period bounds the claim window. Code: Y - implements FST_DT for medical, FILL_DT for pharmacy, filters to [INDEX_DATE, OBS_END_DT], and deduplicates by (PATID, MED_ABBR, DATE_SERVICE, CLAIM_TYPE). Note: spec uses 'ENDDATE' while code uses 'OBS_END_DT' - these represent the same concept (patient observation end date).</t>
+          <t>Spec: N - Spec says to remove pharmacy claims with DAY_SUPPLY &lt; 1 or missing, but Protocol Section 5.1.2 says 'When pharmacy claims are missing days supply, or when days supply values are anomalous, 28 days will be assumed.' Protocol: Y - Protocol defines 28-day default for anomalous pharmacy DAY_SUPPLY. Code: Y - Code implements the spec's delete behavior (lot_program.R line 3066), which contradicts protocol. NOTE: This is a material protocol-vs-code mismatch. See Row 16 (DAY_SUPPLY anomalous values) for full details. The protocol-correct behavior would be to default to 28 instead of deleting.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Claude Review 2026-03-18</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>No discrepancy found. Aligned with protocol. Minor naming difference: spec references ENDDATE while code uses OBS_END_DT (both represent the patient's observation end date defined as earliest of death, disenrollment, or study end).</t>
+          <t>MATERIAL DISCREPANCY FLAGGED: Protocol Section 5.1.2 says to default anomalous/missing pharmacy DAY_SUPPLY to 28 days. Current spec and code DELETE these claims instead. See Row 16 for detailed analysis. Decision required: align with protocol (default to 28) or document intentional deviation.</t>
         </is>
       </c>
     </row>
@@ -19256,7 +19272,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Binary flag (0 or 1). =1 if (LOT1_TX_AUTO_DT_2 - LOT1_TX_AUTO_DT_1 + 1) &lt;= 180 AND LOT1_TX_AUTO_DT_2 &lt;= ENDDATE AND there is not an ALLO SCT such that LOT1_TX_AUTO_DT_1 &lt;= TX_ALLO{i} &lt;= LOT1_TX_AUTO_DT_2. Else = 0. A planned tandem SCT is two autologous SCTs &gt;=60 to &lt;=180 days apart with no intervening allogeneic SCT.</t>
+          <t>Binary flag (0 or 1). =1 if (LOT1_TX_AUTO_DT_2 - LOT1_TX_AUTO_DT_1 + 1) &gt;= 60 AND (LOT1_TX_AUTO_DT_2 - LOT1_TX_AUTO_DT_1 + 1) &lt;= 180 AND LOT1_TX_AUTO_DT_2 &lt;= ENDDATE AND there is not an ALLO SCT such that LOT1_TX_AUTO_DT_1 &lt;= TX_ALLO{i} &lt;= LOT1_TX_AUTO_DT_2. Else = 0. A planned tandem SCT is two autologous SCTs &gt;=60 to &lt;=180 days apart with no intervening allogeneic SCT. The &gt;=60 day minimum gap is enforced during AUTO SCT date processing (sct_auto_gap_days=60).</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -19276,17 +19292,22 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>YYY</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Spec says '(LOT1_TX_AUTO_DT_2 - LOT1_TX_AUTO_DT_1 + 1) &lt;= 180' which matches code's 'datediff + 1 &lt;= 180'. However, the spec does NOT mention the &gt;=60 day minimum gap between tandem SCTs that the protocol explicitly requires ('&gt;=60 to &lt;=180 days apart'). The code enforces the 60-day gap via the AUTO date processing in Step S13 (sct_auto_gap_days=60), so protocol and code agree but spec omits the &gt;=60 day lower bound.</t>
+          <t>Spec, protocol, and code now all agree. Definition updated to include the &gt;=60 day lower bound from Protocol Section 5 ('&gt;=60 to &lt;=180 days apart'). The 60-day gap is enforced in code (Step S13 sct_auto_gap_days=60).</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Claude Review 2026-03-18</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Partial discrepancy: Spec omits the &gt;=60 day minimum gap between tandem AUTO SCTs. Protocol Section 5 clearly states 'at least two autologous SCTs &gt;=60 to &lt;=180 days apart.' The 60-day gap is enforced in code (Step S13 sct_auto_gap_days=60) but not explicitly stated in the spec's tandem flag definition.</t>
+          <t>RESOLVED: Previously, spec omitted the &gt;=60 day minimum gap between tandem AUTO SCTs. Definition now includes &gt;=60 AND &lt;=180 days per Protocol Section 5 and code (sct_auto_gap_days=60).</t>
         </is>
       </c>
     </row>
@@ -19464,7 +19485,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Date (or missing). Set to min(LOT1_TX_AUTO_DT_1, LOT1_TX_ENDDATE) when at least one exists. If both fields are missing then set to missing. More precisely, this is the earliest SCT of any type (AUTO, ALLO, or CART) occurring during LOT1.</t>
+          <t>Date (or missing). Set to least(LOT1_TX_AUTO_DT_1, FIRST_ALLO_DT, FIRST_CART_DT) when at least one exists. If all three are missing then set to missing. This is the earliest actual SCT event date of any type (AUTO, ALLO, or CART) occurring during LOT1.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -19484,32 +19505,22 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>YYY</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Spec definition says 'Set to min(LOT1_TX_AUTO_DT_1, LOT1_TX_ENDDATE)' which is incomplete. The code and protocol define it as the earliest of AUTO_DT_1, FIRST_ALLO_DT, and FIRST_CART_DT -- not LOT1_TX_ENDDATE. LOT1_TX_ENDDATE is a derived end date (day before the ending event), not the actual SCT date. Protocol and code agree on using actual first SCT dates.</t>
+          <t>Spec, protocol, and code now all agree. Definition corrected from 'min(LOT1_TX_AUTO_DT_1, LOT1_TX_ENDDATE)' to 'least(LOT1_TX_AUTO_DT_1, FIRST_ALLO_DT, FIRST_CART_DT)' per code (lot_program.R lines 3963-3972). LOT1_TX_ENDDATE was incorrect here because it is the day BEFORE an SCT-ending event, not the actual SCT date.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Claude Review 2026-03-18</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Discrepancy found: Spec defines LOT1_1ST_SCT_DT as 'min(LOT1_TX_AUTO_DT_1</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> LOT1_TX_ENDDATE)' but this is incorrect. LOT1_TX_ENDDATE is the day BEFORE an SCT-ending event (i.e. the end date of LOT1 due to SCT) and would be 1 day earlier than the actual SCT. The correct definition per code (line 3963-3972) is min(LOT1_TX_AUTO_DT_1</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> FIRST_ALLO_DT</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> FIRST_CART_DT) which uses the actual SCT dates. The spec should reference FIRST_ALLO_DT and FIRST_CART_DT rather than LOT1_TX_ENDDATE.</t>
+          <t>RESOLVED: Previously used min(LOT1_TX_AUTO_DT_1, LOT1_TX_ENDDATE) which mixed an actual SCT date with a derived end date (day before SCT). Corrected to least(LOT1_TX_AUTO_DT_1, FIRST_ALLO_DT, FIRST_CART_DT) per code lines 3963-3972.</t>
         </is>
       </c>
     </row>

</xml_diff>